<commit_message>
Pay matching Xero bills and attach order details
- plan: fetch unpaid supplier bills and pay the one matching a spend line
  (amount due, date window; bill number or supplier name breaks ties,
  otherwise review). Bills are matched before orders and rules so costs
  are never entered twice.
- plan/apply: treat existing bill payments on the account as "exists",
  alongside spend/receive money.
- apply: create payments for bill rows; attach a text record of the
  marketplace order (items, order link) to itemised transactions.
- Plan CSV gains bill_id and order_url columns; older plans still load.
- Parse Xero's legacy /Date(ms)/ values.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YCVrrsKS5fzm9RMdyPCBPm
</commit_message>
<xml_diff>
--- a/internal/reconcile/testdata/ebay.xlsx
+++ b/internal/reconcile/testdata/ebay.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,11 @@
           <t>OrderTotal</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Order Details</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -505,6 +510,11 @@
           <t>£8.99</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=11-11111-11111</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -548,6 +558,11 @@
           <t>£74.81</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=22-22222-22222</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -591,6 +606,11 @@
           <t>£39.64</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=33-33333-33333</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -634,6 +654,11 @@
           <t>£39.64</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=33-33333-33333</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -677,6 +702,11 @@
           <t>£0.00</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=44-44444-44444</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -720,6 +750,11 @@
           <t>£15.00</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=55-55555-55555</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -761,6 +796,11 @@
       <c r="I8" t="inlineStr">
         <is>
           <t>£15.00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://order.ebay.co.uk/ord/show?orderId=55-55555-55555</t>
         </is>
       </c>
     </row>

</xml_diff>